<commit_message>
Undo last entry — Antelias
</commit_message>
<xml_diff>
--- a/data/antelias.xlsx
+++ b/data/antelias.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,38 +485,6 @@
           <t>Note</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-08 03:30</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>lumber for framing</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -529,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -554,32 +522,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>September</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Year Total</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>